<commit_message>
Clarify workbook grouping template
</commit_message>
<xml_diff>
--- a/templates/dataset-analyzer-template.xlsx
+++ b/templates/dataset-analyzer-template.xlsx
@@ -7,13 +7,189 @@
     <sheet sheetId="1" name="Data" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Groups" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Variables" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Instructions" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Case #
+Unit: -
+GroupKey: test_inputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Gross Weight
+Unit: lb
+GroupKey: test_inputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Pressure Altitude
+Unit: ft
+GroupKey: test_inputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: OAT
+Unit: °C
+GroupKey: test_inputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: VR Exp
+Unit: kt
+GroupKey: expected_outputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: V2 Exp
+Unit: kt
+GroupKey: expected_outputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: TO Dist Exp
+Unit: m
+GroupKey: expected_outputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: VR Act
+Unit: kt
+GroupKey: actual_outputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: V2 Act
+Unit: kt
+GroupKey: actual_outputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: TO Dist Act
+Unit: m
+GroupKey: actual_outputs
+DataType: number</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Flaps Setting
+Unit: -
+GroupKey: inputs
+DataType: string</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Runway Condition
+Unit: -
+GroupKey: inputs
+DataType: string</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Anti-Ice
+Unit: -
+GroupKey: inputs
+DataType: string</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Notes
+Unit: -
+GroupKey: logged_data
+DataType: string</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Display: Pass/Fail
+Unit: -
+GroupKey: logged_data
+DataType: string</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="107">
+  <si>
+    <t>Test Inputs</t>
+  </si>
+  <si>
+    <t>Expected Outputs</t>
+  </si>
+  <si>
+    <t>Actual Outputs</t>
+  </si>
+  <si>
+    <t>Inputs</t>
+  </si>
+  <si>
+    <t>Logged Data</t>
+  </si>
   <si>
     <t>Case</t>
   </si>
@@ -93,9 +269,6 @@
     <t>test_inputs</t>
   </si>
   <si>
-    <t>Test Inputs</t>
-  </si>
-  <si>
     <t>#2f8cff</t>
   </si>
   <si>
@@ -105,18 +278,12 @@
     <t>expected_outputs</t>
   </si>
   <si>
-    <t>Expected Outputs</t>
-  </si>
-  <si>
     <t>#39b54a</t>
   </si>
   <si>
     <t>actual_outputs</t>
   </si>
   <si>
-    <t>Actual Outputs</t>
-  </si>
-  <si>
     <t>#9b5de5</t>
   </si>
   <si>
@@ -150,18 +317,12 @@
     <t>inputs</t>
   </si>
   <si>
-    <t>Inputs</t>
-  </si>
-  <si>
     <t>#4169e1</t>
   </si>
   <si>
     <t>logged_data</t>
   </si>
   <si>
-    <t>Logged Data</t>
-  </si>
-  <si>
     <t>#c43ac4</t>
   </si>
   <si>
@@ -298,13 +459,49 @@
   </si>
   <si>
     <t>Pass/Fail</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>The app groups Data columns using metadata, not by reading visual merged cells.</t>
+  </si>
+  <si>
+    <t>Data row 1</t>
+  </si>
+  <si>
+    <t>Visual group headers only. They help humans see the grouping in Excel.</t>
+  </si>
+  <si>
+    <t>Data row 2</t>
+  </si>
+  <si>
+    <t>Machine-readable VariableKey headers. These must match Variables.VariableKey.</t>
+  </si>
+  <si>
+    <t>Groups sheet</t>
+  </si>
+  <si>
+    <t>Defines GroupKey, display name, color, order, and default visibility.</t>
+  </si>
+  <si>
+    <t>Variables sheet</t>
+  </si>
+  <si>
+    <t>Maps every Data column to a GroupKey and declares label, unit, type, order, visibility, and source.</t>
+  </si>
+  <si>
+    <t>Custom data</t>
+  </si>
+  <si>
+    <t>Add your own groups and variables here. Every variable you want displayed must be listed in Variables.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -314,14 +511,63 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F8CFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF39B54A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9B5DE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4169E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC43AC4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEEAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6A600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7A00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B8C8"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -336,9 +582,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,7 +948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -688,197 +958,233 @@
     <col min="13" max="15" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="O1" s="5"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="E2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="F2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="G2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="H2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="I2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="J2" s="6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>65000</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>16.6</v>
-      </c>
-      <c r="E2">
-        <v>120</v>
-      </c>
-      <c r="F2">
-        <v>130.5</v>
-      </c>
-      <c r="G2">
-        <v>980</v>
-      </c>
-      <c r="H2">
-        <v>120</v>
-      </c>
-      <c r="I2">
-        <v>131.1</v>
-      </c>
-      <c r="J2">
-        <v>994</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="K2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3">
-        <v>65300</v>
+        <v>65000</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>16.9</v>
+        <v>16.6</v>
       </c>
       <c r="E3">
-        <v>120.4</v>
+        <v>120</v>
       </c>
       <c r="F3">
-        <v>130.9</v>
+        <v>130.5</v>
       </c>
       <c r="G3">
-        <v>1025</v>
+        <v>980</v>
       </c>
       <c r="H3">
-        <v>120.6</v>
+        <v>120</v>
       </c>
       <c r="I3">
-        <v>131.4</v>
+        <v>131.1</v>
       </c>
       <c r="J3">
-        <v>1043</v>
+        <v>994</v>
       </c>
       <c r="K3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="L3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="M3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="O3" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
-        <v>65550</v>
+        <v>65300</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
+        <v>16.9</v>
+      </c>
+      <c r="E4">
+        <v>120.4</v>
+      </c>
+      <c r="F4">
+        <v>130.9</v>
+      </c>
+      <c r="G4">
+        <v>1025</v>
+      </c>
+      <c r="H4">
+        <v>120.6</v>
+      </c>
+      <c r="I4">
+        <v>131.4</v>
+      </c>
+      <c r="J4">
+        <v>1043</v>
+      </c>
+      <c r="K4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M4" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>65550</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
         <v>17</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>120.8</v>
       </c>
-      <c r="F4">
+      <c r="F5">
         <v>131.4</v>
       </c>
-      <c r="G4">
+      <c r="G5">
         <v>1065</v>
       </c>
-      <c r="H4">
+      <c r="H5">
         <v>121.1</v>
       </c>
-      <c r="I4">
+      <c r="I5">
         <v>131.8</v>
       </c>
-      <c r="J4">
+      <c r="J5">
         <v>1085</v>
       </c>
-      <c r="K4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L4" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O4" t="s">
-        <v>19</v>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" t="s">
+        <v>22</v>
+      </c>
+      <c r="N5" t="s">
+        <v>23</v>
+      </c>
+      <c r="O5" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:O5"/>
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:O1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -894,157 +1200,157 @@
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>24</v>
+    <row r="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
+        <v>0</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="D2">
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
+        <v>1</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>34</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" t="s">
-        <v>34</v>
+        <v>2</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="D4">
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>39</v>
       </c>
       <c r="D5">
         <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="D6">
         <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>45</v>
       </c>
       <c r="D7">
         <v>60</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" t="s">
-        <v>46</v>
+        <v>3</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>47</v>
       </c>
       <c r="D8">
         <v>70</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>49</v>
       </c>
       <c r="D9">
         <v>80</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1067,44 +1373,44 @@
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="B1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
         <v>55</v>
@@ -1113,7 +1419,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H2" t="s">
         <v>56</v>
@@ -1121,13 +1427,13 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
         <v>58</v>
@@ -1139,7 +1445,7 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H3" t="s">
         <v>56</v>
@@ -1147,13 +1453,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
         <v>60</v>
@@ -1165,7 +1471,7 @@
         <v>20</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
         <v>56</v>
@@ -1173,13 +1479,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
         <v>61</v>
@@ -1191,7 +1497,7 @@
         <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H5" t="s">
         <v>56</v>
@@ -1199,13 +1505,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
         <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
         <v>63</v>
@@ -1217,7 +1523,7 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H6" t="s">
         <v>56</v>
@@ -1225,13 +1531,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>64</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
         <v>63</v>
@@ -1243,7 +1549,7 @@
         <v>20</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H7" t="s">
         <v>56</v>
@@ -1251,13 +1557,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
         <v>65</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
         <v>66</v>
@@ -1269,7 +1575,7 @@
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H8" t="s">
         <v>56</v>
@@ -1277,13 +1583,13 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
         <v>67</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
         <v>63</v>
@@ -1295,7 +1601,7 @@
         <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H9" t="s">
         <v>56</v>
@@ -1303,13 +1609,13 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
         <v>68</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
         <v>63</v>
@@ -1321,7 +1627,7 @@
         <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H10" t="s">
         <v>56</v>
@@ -1329,13 +1635,13 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
         <v>66</v>
@@ -1347,7 +1653,7 @@
         <v>30</v>
       </c>
       <c r="G11" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H11" t="s">
         <v>56</v>
@@ -1361,7 +1667,7 @@
         <v>71</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
         <v>63</v>
@@ -1373,7 +1679,7 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H12" t="s">
         <v>72</v>
@@ -1387,7 +1693,7 @@
         <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
         <v>63</v>
@@ -1399,7 +1705,7 @@
         <v>20</v>
       </c>
       <c r="G13" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H13" t="s">
         <v>72</v>
@@ -1413,7 +1719,7 @@
         <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
         <v>66</v>
@@ -1425,7 +1731,7 @@
         <v>30</v>
       </c>
       <c r="G14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H14" t="s">
         <v>72</v>
@@ -1439,7 +1745,7 @@
         <v>78</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D15" t="s">
         <v>63</v>
@@ -1451,7 +1757,7 @@
         <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H15" t="s">
         <v>72</v>
@@ -1465,7 +1771,7 @@
         <v>80</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D16" t="s">
         <v>63</v>
@@ -1477,7 +1783,7 @@
         <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H16" t="s">
         <v>72</v>
@@ -1491,7 +1797,7 @@
         <v>82</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
         <v>66</v>
@@ -1503,7 +1809,7 @@
         <v>30</v>
       </c>
       <c r="G17" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H17" t="s">
         <v>72</v>
@@ -1517,7 +1823,7 @@
         <v>84</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D18" t="s">
         <v>85</v>
@@ -1529,7 +1835,7 @@
         <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H18" t="s">
         <v>72</v>
@@ -1543,7 +1849,7 @@
         <v>87</v>
       </c>
       <c r="C19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D19" t="s">
         <v>85</v>
@@ -1555,7 +1861,7 @@
         <v>20</v>
       </c>
       <c r="G19" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H19" t="s">
         <v>72</v>
@@ -1569,7 +1875,7 @@
         <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D20" t="s">
         <v>85</v>
@@ -1581,7 +1887,7 @@
         <v>30</v>
       </c>
       <c r="G20" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H20" t="s">
         <v>72</v>
@@ -1589,16 +1895,16 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B21" t="s">
         <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E21" t="s">
         <v>91</v>
@@ -1607,7 +1913,7 @@
         <v>10</v>
       </c>
       <c r="G21" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H21" t="s">
         <v>56</v>
@@ -1615,16 +1921,16 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B22" t="s">
         <v>92</v>
       </c>
       <c r="C22" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D22" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E22" t="s">
         <v>91</v>
@@ -1633,7 +1939,7 @@
         <v>20</v>
       </c>
       <c r="G22" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H22" t="s">
         <v>56</v>
@@ -1641,16 +1947,16 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
         <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D23" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E23" t="s">
         <v>91</v>
@@ -1659,7 +1965,7 @@
         <v>30</v>
       </c>
       <c r="G23" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H23" t="s">
         <v>56</v>
@@ -1667,16 +1973,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B24" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C24" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D24" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E24" t="s">
         <v>91</v>
@@ -1685,7 +1991,7 @@
         <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H24" t="s">
         <v>56</v>
@@ -1693,16 +1999,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B25" t="s">
         <v>94</v>
       </c>
       <c r="C25" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s">
         <v>91</v>
@@ -1711,10 +2017,73 @@
         <v>20</v>
       </c>
       <c r="G25" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H25" t="s">
         <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>